<commit_message>
Mejora flujo SurveyMonkey y validación analítica
</commit_message>
<xml_diff>
--- a/api/tests/testthat/fixtures/surveymonkey/golden/Administrativo_inst.xlsx
+++ b/api/tests/testthat/fixtures/surveymonkey/golden/Administrativo_inst.xlsx
@@ -470,7 +470,7 @@
     <t xml:space="preserve">es</t>
   </si>
   <si>
-    <t xml:space="preserve">20260502</t>
+    <t xml:space="preserve">20260523</t>
   </si>
   <si>
     <t xml:space="preserve">order</t>
@@ -1021,11 +1021,21 @@
       <c r="C2" t="s">
         <v>11</v>
       </c>
-      <c r="D2"/>
-      <c r="E2"/>
-      <c r="F2"/>
-      <c r="G2"/>
-      <c r="H2"/>
+      <c r="D2" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E2" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F2" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G2" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H2" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I2" t="s">
         <v>10</v>
       </c>
@@ -1040,11 +1050,21 @@
       <c r="C3" t="s">
         <v>13</v>
       </c>
-      <c r="D3"/>
-      <c r="E3"/>
-      <c r="F3"/>
-      <c r="G3"/>
-      <c r="H3"/>
+      <c r="D3" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E3" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F3" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G3" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H3" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I3" t="s">
         <v>10</v>
       </c>
@@ -1053,13 +1073,27 @@
       <c r="A4" t="s">
         <v>14</v>
       </c>
-      <c r="B4"/>
-      <c r="C4"/>
-      <c r="D4"/>
-      <c r="E4"/>
-      <c r="F4"/>
-      <c r="G4"/>
-      <c r="H4"/>
+      <c r="B4" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="C4" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="D4" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E4" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F4" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G4" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H4" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I4" t="s">
         <v>10</v>
       </c>
@@ -1074,11 +1108,21 @@
       <c r="C5" t="s">
         <v>17</v>
       </c>
-      <c r="D5"/>
-      <c r="E5"/>
-      <c r="F5"/>
-      <c r="G5"/>
-      <c r="H5"/>
+      <c r="D5" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E5" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F5" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G5" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H5" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I5" t="s">
         <v>18</v>
       </c>
@@ -1093,11 +1137,21 @@
       <c r="C6" t="s">
         <v>20</v>
       </c>
-      <c r="D6"/>
-      <c r="E6"/>
-      <c r="F6"/>
-      <c r="G6"/>
-      <c r="H6"/>
+      <c r="D6" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E6" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F6" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G6" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H6" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I6" t="s">
         <v>19</v>
       </c>
@@ -1112,11 +1166,21 @@
       <c r="C7" t="s">
         <v>23</v>
       </c>
-      <c r="D7"/>
-      <c r="E7"/>
-      <c r="F7"/>
-      <c r="G7"/>
-      <c r="H7"/>
+      <c r="D7" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E7" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F7" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G7" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H7" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I7" t="s">
         <v>19</v>
       </c>
@@ -1125,13 +1189,27 @@
       <c r="A8" t="s">
         <v>14</v>
       </c>
-      <c r="B8"/>
-      <c r="C8"/>
-      <c r="D8"/>
-      <c r="E8"/>
-      <c r="F8"/>
-      <c r="G8"/>
-      <c r="H8"/>
+      <c r="B8" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="C8" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="D8" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E8" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F8" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G8" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H8" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I8" t="s">
         <v>19</v>
       </c>
@@ -1146,11 +1224,21 @@
       <c r="C9" t="s">
         <v>26</v>
       </c>
-      <c r="D9"/>
-      <c r="E9"/>
-      <c r="F9"/>
-      <c r="G9"/>
-      <c r="H9"/>
+      <c r="D9" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E9" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F9" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G9" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H9" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I9" t="s">
         <v>18</v>
       </c>
@@ -1165,11 +1253,21 @@
       <c r="C10" t="s">
         <v>28</v>
       </c>
-      <c r="D10"/>
-      <c r="E10"/>
-      <c r="F10"/>
-      <c r="G10"/>
-      <c r="H10"/>
+      <c r="D10" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E10" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F10" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G10" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H10" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I10" t="s">
         <v>18</v>
       </c>
@@ -1184,11 +1282,21 @@
       <c r="C11" t="s">
         <v>30</v>
       </c>
-      <c r="D11"/>
-      <c r="E11"/>
-      <c r="F11"/>
-      <c r="G11"/>
-      <c r="H11"/>
+      <c r="D11" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E11" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F11" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G11" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H11" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I11" t="s">
         <v>31</v>
       </c>
@@ -1203,11 +1311,21 @@
       <c r="C12" t="s">
         <v>30</v>
       </c>
-      <c r="D12"/>
-      <c r="E12"/>
-      <c r="F12"/>
-      <c r="G12"/>
-      <c r="H12"/>
+      <c r="D12" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E12" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F12" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G12" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H12" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I12" t="s">
         <v>31</v>
       </c>
@@ -1222,11 +1340,21 @@
       <c r="C13" t="s">
         <v>34</v>
       </c>
-      <c r="D13"/>
-      <c r="E13"/>
-      <c r="F13"/>
-      <c r="G13"/>
-      <c r="H13"/>
+      <c r="D13" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E13" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F13" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G13" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H13" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I13" t="s">
         <v>31</v>
       </c>
@@ -1241,11 +1369,21 @@
       <c r="C14" t="s">
         <v>36</v>
       </c>
-      <c r="D14"/>
-      <c r="E14"/>
-      <c r="F14"/>
-      <c r="G14"/>
-      <c r="H14"/>
+      <c r="D14" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E14" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F14" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G14" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H14" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I14" t="s">
         <v>31</v>
       </c>
@@ -1254,13 +1392,27 @@
       <c r="A15" t="s">
         <v>14</v>
       </c>
-      <c r="B15"/>
-      <c r="C15"/>
-      <c r="D15"/>
-      <c r="E15"/>
-      <c r="F15"/>
-      <c r="G15"/>
-      <c r="H15"/>
+      <c r="B15" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="C15" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="D15" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E15" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F15" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G15" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H15" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I15" t="s">
         <v>31</v>
       </c>
@@ -1275,11 +1427,21 @@
       <c r="C16" t="s">
         <v>39</v>
       </c>
-      <c r="D16"/>
-      <c r="E16"/>
-      <c r="F16"/>
-      <c r="G16"/>
-      <c r="H16"/>
+      <c r="D16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H16" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I16" t="s">
         <v>18</v>
       </c>
@@ -1291,12 +1453,24 @@
       <c r="B17" t="s">
         <v>40</v>
       </c>
-      <c r="C17"/>
-      <c r="D17"/>
-      <c r="E17"/>
-      <c r="F17"/>
-      <c r="G17"/>
-      <c r="H17"/>
+      <c r="C17" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="D17" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E17" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F17" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G17" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H17" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I17" t="s">
         <v>41</v>
       </c>
@@ -1311,11 +1485,21 @@
       <c r="C18" t="s">
         <v>44</v>
       </c>
-      <c r="D18"/>
-      <c r="E18"/>
-      <c r="F18"/>
-      <c r="G18"/>
-      <c r="H18"/>
+      <c r="D18" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E18" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F18" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G18" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H18" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I18" t="s">
         <v>41</v>
       </c>
@@ -1330,11 +1514,21 @@
       <c r="C19" t="s">
         <v>46</v>
       </c>
-      <c r="D19"/>
-      <c r="E19"/>
-      <c r="F19"/>
-      <c r="G19"/>
-      <c r="H19"/>
+      <c r="D19" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E19" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F19" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G19" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H19" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I19" t="s">
         <v>41</v>
       </c>
@@ -1349,11 +1543,21 @@
       <c r="C20" t="s">
         <v>48</v>
       </c>
-      <c r="D20"/>
-      <c r="E20"/>
-      <c r="F20"/>
-      <c r="G20"/>
-      <c r="H20"/>
+      <c r="D20" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E20" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F20" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G20" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H20" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I20" t="s">
         <v>41</v>
       </c>
@@ -1362,13 +1566,27 @@
       <c r="A21" t="s">
         <v>14</v>
       </c>
-      <c r="B21"/>
-      <c r="C21"/>
-      <c r="D21"/>
-      <c r="E21"/>
-      <c r="F21"/>
-      <c r="G21"/>
-      <c r="H21"/>
+      <c r="B21" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="C21" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="D21" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E21" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F21" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G21" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H21" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I21" t="s">
         <v>41</v>
       </c>
@@ -1380,12 +1598,24 @@
       <c r="B22" t="s">
         <v>49</v>
       </c>
-      <c r="C22"/>
-      <c r="D22"/>
-      <c r="E22"/>
-      <c r="F22"/>
-      <c r="G22"/>
-      <c r="H22"/>
+      <c r="C22" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="D22" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E22" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F22" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G22" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H22" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I22" t="s">
         <v>50</v>
       </c>
@@ -1400,11 +1630,21 @@
       <c r="C23" t="s">
         <v>52</v>
       </c>
-      <c r="D23"/>
-      <c r="E23"/>
-      <c r="F23"/>
-      <c r="G23"/>
-      <c r="H23"/>
+      <c r="D23" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E23" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F23" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G23" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H23" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I23" t="s">
         <v>50</v>
       </c>
@@ -1419,11 +1659,21 @@
       <c r="C24" t="s">
         <v>54</v>
       </c>
-      <c r="D24"/>
-      <c r="E24"/>
-      <c r="F24"/>
-      <c r="G24"/>
-      <c r="H24"/>
+      <c r="D24" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E24" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F24" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G24" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H24" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I24" t="s">
         <v>50</v>
       </c>
@@ -1438,11 +1688,21 @@
       <c r="C25" t="s">
         <v>56</v>
       </c>
-      <c r="D25"/>
-      <c r="E25"/>
-      <c r="F25"/>
-      <c r="G25"/>
-      <c r="H25"/>
+      <c r="D25" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E25" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F25" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G25" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H25" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I25" t="s">
         <v>50</v>
       </c>
@@ -1457,11 +1717,21 @@
       <c r="C26" t="s">
         <v>58</v>
       </c>
-      <c r="D26"/>
-      <c r="E26"/>
-      <c r="F26"/>
-      <c r="G26"/>
-      <c r="H26"/>
+      <c r="D26" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E26" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F26" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G26" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H26" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I26" t="s">
         <v>50</v>
       </c>
@@ -1476,11 +1746,21 @@
       <c r="C27" t="s">
         <v>60</v>
       </c>
-      <c r="D27"/>
-      <c r="E27"/>
-      <c r="F27"/>
-      <c r="G27"/>
-      <c r="H27"/>
+      <c r="D27" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E27" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F27" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G27" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H27" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I27" t="s">
         <v>50</v>
       </c>
@@ -1495,11 +1775,21 @@
       <c r="C28" t="s">
         <v>62</v>
       </c>
-      <c r="D28"/>
-      <c r="E28"/>
-      <c r="F28"/>
-      <c r="G28"/>
-      <c r="H28"/>
+      <c r="D28" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E28" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F28" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G28" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H28" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I28" t="s">
         <v>50</v>
       </c>
@@ -1514,11 +1804,21 @@
       <c r="C29" t="s">
         <v>64</v>
       </c>
-      <c r="D29"/>
-      <c r="E29"/>
-      <c r="F29"/>
-      <c r="G29"/>
-      <c r="H29"/>
+      <c r="D29" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E29" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F29" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G29" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H29" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I29" t="s">
         <v>50</v>
       </c>
@@ -1527,13 +1827,27 @@
       <c r="A30" t="s">
         <v>14</v>
       </c>
-      <c r="B30"/>
-      <c r="C30"/>
-      <c r="D30"/>
-      <c r="E30"/>
-      <c r="F30"/>
-      <c r="G30"/>
-      <c r="H30"/>
+      <c r="B30" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="C30" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="D30" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E30" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F30" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G30" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H30" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I30" t="s">
         <v>50</v>
       </c>
@@ -1545,12 +1859,24 @@
       <c r="B31" t="s">
         <v>65</v>
       </c>
-      <c r="C31"/>
-      <c r="D31"/>
-      <c r="E31"/>
-      <c r="F31"/>
-      <c r="G31"/>
-      <c r="H31"/>
+      <c r="C31" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="D31" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E31" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F31" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G31" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H31" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I31" t="s">
         <v>66</v>
       </c>
@@ -1565,11 +1891,21 @@
       <c r="C32" t="s">
         <v>68</v>
       </c>
-      <c r="D32"/>
-      <c r="E32"/>
-      <c r="F32"/>
-      <c r="G32"/>
-      <c r="H32"/>
+      <c r="D32" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E32" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F32" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G32" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H32" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I32" t="s">
         <v>66</v>
       </c>
@@ -1584,11 +1920,21 @@
       <c r="C33" t="s">
         <v>70</v>
       </c>
-      <c r="D33"/>
-      <c r="E33"/>
-      <c r="F33"/>
-      <c r="G33"/>
-      <c r="H33"/>
+      <c r="D33" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E33" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F33" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G33" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H33" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I33" t="s">
         <v>66</v>
       </c>
@@ -1603,11 +1949,21 @@
       <c r="C34" t="s">
         <v>72</v>
       </c>
-      <c r="D34"/>
-      <c r="E34"/>
-      <c r="F34"/>
-      <c r="G34"/>
-      <c r="H34"/>
+      <c r="D34" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E34" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F34" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G34" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H34" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I34" t="s">
         <v>66</v>
       </c>
@@ -1622,11 +1978,21 @@
       <c r="C35" t="s">
         <v>74</v>
       </c>
-      <c r="D35"/>
-      <c r="E35"/>
-      <c r="F35"/>
-      <c r="G35"/>
-      <c r="H35"/>
+      <c r="D35" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E35" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F35" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G35" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H35" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I35" t="s">
         <v>66</v>
       </c>
@@ -1641,11 +2007,21 @@
       <c r="C36" t="s">
         <v>76</v>
       </c>
-      <c r="D36"/>
-      <c r="E36"/>
-      <c r="F36"/>
-      <c r="G36"/>
-      <c r="H36"/>
+      <c r="D36" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E36" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F36" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G36" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H36" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I36" t="s">
         <v>66</v>
       </c>
@@ -1660,11 +2036,21 @@
       <c r="C37" t="s">
         <v>78</v>
       </c>
-      <c r="D37"/>
-      <c r="E37"/>
-      <c r="F37"/>
-      <c r="G37"/>
-      <c r="H37"/>
+      <c r="D37" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E37" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F37" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G37" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H37" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I37" t="s">
         <v>66</v>
       </c>
@@ -1679,11 +2065,21 @@
       <c r="C38" t="s">
         <v>80</v>
       </c>
-      <c r="D38"/>
-      <c r="E38"/>
-      <c r="F38"/>
-      <c r="G38"/>
-      <c r="H38"/>
+      <c r="D38" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E38" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F38" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G38" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H38" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I38" t="s">
         <v>66</v>
       </c>
@@ -1698,11 +2094,21 @@
       <c r="C39" t="s">
         <v>82</v>
       </c>
-      <c r="D39"/>
-      <c r="E39"/>
-      <c r="F39"/>
-      <c r="G39"/>
-      <c r="H39"/>
+      <c r="D39" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E39" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F39" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G39" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H39" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I39" t="s">
         <v>66</v>
       </c>
@@ -1711,13 +2117,27 @@
       <c r="A40" t="s">
         <v>14</v>
       </c>
-      <c r="B40"/>
-      <c r="C40"/>
-      <c r="D40"/>
-      <c r="E40"/>
-      <c r="F40"/>
-      <c r="G40"/>
-      <c r="H40"/>
+      <c r="B40" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="C40" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="D40" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E40" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F40" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G40" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H40" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I40" t="s">
         <v>66</v>
       </c>
@@ -1729,12 +2149,24 @@
       <c r="B41" t="s">
         <v>83</v>
       </c>
-      <c r="C41"/>
-      <c r="D41"/>
-      <c r="E41"/>
-      <c r="F41"/>
-      <c r="G41"/>
-      <c r="H41"/>
+      <c r="C41" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="D41" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E41" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F41" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G41" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H41" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I41" t="s">
         <v>84</v>
       </c>
@@ -1749,11 +2181,21 @@
       <c r="C42" t="s">
         <v>86</v>
       </c>
-      <c r="D42"/>
-      <c r="E42"/>
-      <c r="F42"/>
-      <c r="G42"/>
-      <c r="H42"/>
+      <c r="D42" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E42" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F42" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G42" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H42" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I42" t="s">
         <v>84</v>
       </c>
@@ -1768,11 +2210,21 @@
       <c r="C43" t="s">
         <v>88</v>
       </c>
-      <c r="D43"/>
-      <c r="E43"/>
-      <c r="F43"/>
-      <c r="G43"/>
-      <c r="H43"/>
+      <c r="D43" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E43" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F43" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G43" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H43" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I43" t="s">
         <v>84</v>
       </c>
@@ -1787,11 +2239,21 @@
       <c r="C44" t="s">
         <v>90</v>
       </c>
-      <c r="D44"/>
-      <c r="E44"/>
-      <c r="F44"/>
-      <c r="G44"/>
-      <c r="H44"/>
+      <c r="D44" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E44" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F44" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G44" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H44" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I44" t="s">
         <v>84</v>
       </c>
@@ -1800,13 +2262,27 @@
       <c r="A45" t="s">
         <v>14</v>
       </c>
-      <c r="B45"/>
-      <c r="C45"/>
-      <c r="D45"/>
-      <c r="E45"/>
-      <c r="F45"/>
-      <c r="G45"/>
-      <c r="H45"/>
+      <c r="B45" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="C45" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="D45" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E45" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F45" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G45" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H45" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I45" t="s">
         <v>84</v>
       </c>
@@ -1818,12 +2294,24 @@
       <c r="B46" t="s">
         <v>91</v>
       </c>
-      <c r="C46"/>
-      <c r="D46"/>
-      <c r="E46"/>
-      <c r="F46"/>
-      <c r="G46"/>
-      <c r="H46"/>
+      <c r="C46" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="D46" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E46" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F46" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G46" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H46" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I46" t="s">
         <v>92</v>
       </c>
@@ -1838,11 +2326,21 @@
       <c r="C47" t="s">
         <v>94</v>
       </c>
-      <c r="D47"/>
-      <c r="E47"/>
-      <c r="F47"/>
-      <c r="G47"/>
-      <c r="H47"/>
+      <c r="D47" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E47" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F47" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G47" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H47" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I47" t="s">
         <v>92</v>
       </c>
@@ -1857,11 +2355,21 @@
       <c r="C48" t="s">
         <v>96</v>
       </c>
-      <c r="D48"/>
-      <c r="E48"/>
-      <c r="F48"/>
-      <c r="G48"/>
-      <c r="H48"/>
+      <c r="D48" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E48" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F48" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G48" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H48" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I48" t="s">
         <v>92</v>
       </c>
@@ -1876,11 +2384,21 @@
       <c r="C49" t="s">
         <v>98</v>
       </c>
-      <c r="D49"/>
-      <c r="E49"/>
-      <c r="F49"/>
-      <c r="G49"/>
-      <c r="H49"/>
+      <c r="D49" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E49" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F49" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G49" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H49" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I49" t="s">
         <v>92</v>
       </c>
@@ -1895,11 +2413,21 @@
       <c r="C50" t="s">
         <v>100</v>
       </c>
-      <c r="D50"/>
-      <c r="E50"/>
-      <c r="F50"/>
-      <c r="G50"/>
-      <c r="H50"/>
+      <c r="D50" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E50" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F50" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G50" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H50" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I50" t="s">
         <v>92</v>
       </c>
@@ -1914,11 +2442,21 @@
       <c r="C51" t="s">
         <v>102</v>
       </c>
-      <c r="D51"/>
-      <c r="E51"/>
-      <c r="F51"/>
-      <c r="G51"/>
-      <c r="H51"/>
+      <c r="D51" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E51" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F51" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G51" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H51" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I51" t="s">
         <v>92</v>
       </c>
@@ -1927,13 +2465,27 @@
       <c r="A52" t="s">
         <v>14</v>
       </c>
-      <c r="B52"/>
-      <c r="C52"/>
-      <c r="D52"/>
-      <c r="E52"/>
-      <c r="F52"/>
-      <c r="G52"/>
-      <c r="H52"/>
+      <c r="B52" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="C52" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="D52" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E52" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F52" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G52" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H52" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I52" t="s">
         <v>92</v>
       </c>
@@ -1948,11 +2500,21 @@
       <c r="C53" t="s">
         <v>20</v>
       </c>
-      <c r="D53"/>
-      <c r="E53"/>
-      <c r="F53"/>
-      <c r="G53"/>
-      <c r="H53"/>
+      <c r="D53" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E53" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F53" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G53" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H53" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I53" t="s">
         <v>19</v>
       </c>
@@ -1967,11 +2529,21 @@
       <c r="C54" t="s">
         <v>105</v>
       </c>
-      <c r="D54"/>
-      <c r="E54"/>
-      <c r="F54"/>
-      <c r="G54"/>
-      <c r="H54"/>
+      <c r="D54" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E54" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F54" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G54" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H54" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I54" t="s">
         <v>19</v>
       </c>
@@ -1986,11 +2558,21 @@
       <c r="C55" t="s">
         <v>108</v>
       </c>
-      <c r="D55"/>
-      <c r="E55"/>
-      <c r="F55"/>
-      <c r="G55"/>
-      <c r="H55"/>
+      <c r="D55" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E55" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F55" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G55" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H55" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I55" t="s">
         <v>19</v>
       </c>
@@ -1999,13 +2581,27 @@
       <c r="A56" t="s">
         <v>14</v>
       </c>
-      <c r="B56"/>
-      <c r="C56"/>
-      <c r="D56"/>
-      <c r="E56"/>
-      <c r="F56"/>
-      <c r="G56"/>
-      <c r="H56"/>
+      <c r="B56" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="C56" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="D56" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="E56" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="F56" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="G56" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="H56" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="I56" t="s">
         <v>19</v>
       </c>
@@ -2408,7 +3004,9 @@
       <c r="H2" t="s">
         <v>12</v>
       </c>
-      <c r="I2"/>
+      <c r="I2" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="J2" t="s">
         <v>10</v>
       </c>
@@ -2433,8 +3031,12 @@
       <c r="Q2" t="s">
         <v>172</v>
       </c>
-      <c r="R2"/>
-      <c r="S2"/>
+      <c r="R2" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S2" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -2488,8 +3090,12 @@
       <c r="Q3" t="s">
         <v>175</v>
       </c>
-      <c r="R3"/>
-      <c r="S3"/>
+      <c r="R3" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S3" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -2543,8 +3149,12 @@
       <c r="Q4" t="s">
         <v>172</v>
       </c>
-      <c r="R4"/>
-      <c r="S4"/>
+      <c r="R4" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S4" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -2571,7 +3181,9 @@
       <c r="H5" t="s">
         <v>24</v>
       </c>
-      <c r="I5"/>
+      <c r="I5" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="J5" t="s">
         <v>18</v>
       </c>
@@ -2596,8 +3208,12 @@
       <c r="Q5" t="s">
         <v>177</v>
       </c>
-      <c r="R5"/>
-      <c r="S5"/>
+      <c r="R5" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S5" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -2624,7 +3240,9 @@
       <c r="H6" t="s">
         <v>24</v>
       </c>
-      <c r="I6"/>
+      <c r="I6" t="e">
+        <v>#N/A</v>
+      </c>
       <c r="J6" t="s">
         <v>18</v>
       </c>
@@ -2649,8 +3267,12 @@
       <c r="Q6" t="s">
         <v>177</v>
       </c>
-      <c r="R6"/>
-      <c r="S6"/>
+      <c r="R6" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S6" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -2704,8 +3326,12 @@
       <c r="Q7" t="s">
         <v>175</v>
       </c>
-      <c r="R7"/>
-      <c r="S7"/>
+      <c r="R7" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S7" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -2759,8 +3385,12 @@
       <c r="Q8" t="s">
         <v>175</v>
       </c>
-      <c r="R8"/>
-      <c r="S8"/>
+      <c r="R8" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S8" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -2814,8 +3444,12 @@
       <c r="Q9" t="s">
         <v>175</v>
       </c>
-      <c r="R9"/>
-      <c r="S9"/>
+      <c r="R9" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S9" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -2869,8 +3503,12 @@
       <c r="Q10" t="s">
         <v>175</v>
       </c>
-      <c r="R10"/>
-      <c r="S10"/>
+      <c r="R10" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S10" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -2924,8 +3562,12 @@
       <c r="Q11" t="s">
         <v>175</v>
       </c>
-      <c r="R11"/>
-      <c r="S11"/>
+      <c r="R11" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S11" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -2979,8 +3621,12 @@
       <c r="Q12" t="s">
         <v>175</v>
       </c>
-      <c r="R12"/>
-      <c r="S12"/>
+      <c r="R12" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S12" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -3034,8 +3680,12 @@
       <c r="Q13" t="s">
         <v>175</v>
       </c>
-      <c r="R13"/>
-      <c r="S13"/>
+      <c r="R13" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S13" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -3089,8 +3739,12 @@
       <c r="Q14" t="s">
         <v>175</v>
       </c>
-      <c r="R14"/>
-      <c r="S14"/>
+      <c r="R14" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S14" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -3144,8 +3798,12 @@
       <c r="Q15" t="s">
         <v>175</v>
       </c>
-      <c r="R15"/>
-      <c r="S15"/>
+      <c r="R15" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S15" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -3199,8 +3857,12 @@
       <c r="Q16" t="s">
         <v>175</v>
       </c>
-      <c r="R16"/>
-      <c r="S16"/>
+      <c r="R16" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S16" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -3254,8 +3916,12 @@
       <c r="Q17" t="s">
         <v>175</v>
       </c>
-      <c r="R17"/>
-      <c r="S17"/>
+      <c r="R17" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S17" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -3309,8 +3975,12 @@
       <c r="Q18" t="s">
         <v>175</v>
       </c>
-      <c r="R18"/>
-      <c r="S18"/>
+      <c r="R18" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S18" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -3364,8 +4034,12 @@
       <c r="Q19" t="s">
         <v>175</v>
       </c>
-      <c r="R19"/>
-      <c r="S19"/>
+      <c r="R19" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S19" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -3419,8 +4093,12 @@
       <c r="Q20" t="s">
         <v>175</v>
       </c>
-      <c r="R20"/>
-      <c r="S20"/>
+      <c r="R20" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S20" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -3474,8 +4152,12 @@
       <c r="Q21" t="s">
         <v>175</v>
       </c>
-      <c r="R21"/>
-      <c r="S21"/>
+      <c r="R21" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S21" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -3529,8 +4211,12 @@
       <c r="Q22" t="s">
         <v>175</v>
       </c>
-      <c r="R22"/>
-      <c r="S22"/>
+      <c r="R22" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S22" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -3584,8 +4270,12 @@
       <c r="Q23" t="s">
         <v>175</v>
       </c>
-      <c r="R23"/>
-      <c r="S23"/>
+      <c r="R23" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S23" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -3639,8 +4329,12 @@
       <c r="Q24" t="s">
         <v>175</v>
       </c>
-      <c r="R24"/>
-      <c r="S24"/>
+      <c r="R24" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S24" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -3694,8 +4388,12 @@
       <c r="Q25" t="s">
         <v>175</v>
       </c>
-      <c r="R25"/>
-      <c r="S25"/>
+      <c r="R25" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S25" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -3749,8 +4447,12 @@
       <c r="Q26" t="s">
         <v>175</v>
       </c>
-      <c r="R26"/>
-      <c r="S26"/>
+      <c r="R26" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S26" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -3804,8 +4506,12 @@
       <c r="Q27" t="s">
         <v>175</v>
       </c>
-      <c r="R27"/>
-      <c r="S27"/>
+      <c r="R27" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S27" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -3859,8 +4565,12 @@
       <c r="Q28" t="s">
         <v>175</v>
       </c>
-      <c r="R28"/>
-      <c r="S28"/>
+      <c r="R28" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S28" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -3914,8 +4624,12 @@
       <c r="Q29" t="s">
         <v>175</v>
       </c>
-      <c r="R29"/>
-      <c r="S29"/>
+      <c r="R29" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S29" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -3969,8 +4683,12 @@
       <c r="Q30" t="s">
         <v>175</v>
       </c>
-      <c r="R30"/>
-      <c r="S30"/>
+      <c r="R30" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S30" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -4024,8 +4742,12 @@
       <c r="Q31" t="s">
         <v>175</v>
       </c>
-      <c r="R31"/>
-      <c r="S31"/>
+      <c r="R31" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S31" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -4079,8 +4801,12 @@
       <c r="Q32" t="s">
         <v>175</v>
       </c>
-      <c r="R32"/>
-      <c r="S32"/>
+      <c r="R32" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S32" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -4134,8 +4860,12 @@
       <c r="Q33" t="s">
         <v>175</v>
       </c>
-      <c r="R33"/>
-      <c r="S33"/>
+      <c r="R33" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S33" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -4189,8 +4919,12 @@
       <c r="Q34" t="s">
         <v>175</v>
       </c>
-      <c r="R34"/>
-      <c r="S34"/>
+      <c r="R34" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S34" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -4244,8 +4978,12 @@
       <c r="Q35" t="s">
         <v>175</v>
       </c>
-      <c r="R35"/>
-      <c r="S35"/>
+      <c r="R35" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S35" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -4299,8 +5037,12 @@
       <c r="Q36" t="s">
         <v>175</v>
       </c>
-      <c r="R36"/>
-      <c r="S36"/>
+      <c r="R36" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S36" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -4354,8 +5096,12 @@
       <c r="Q37" t="s">
         <v>175</v>
       </c>
-      <c r="R37"/>
-      <c r="S37"/>
+      <c r="R37" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S37" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -4409,8 +5155,12 @@
       <c r="Q38" t="s">
         <v>175</v>
       </c>
-      <c r="R38"/>
-      <c r="S38"/>
+      <c r="R38" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="S38" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>